<commit_message>
Atualização semanal do dashboard (dados)
</commit_message>
<xml_diff>
--- a/progresso.xlsx
+++ b/progresso.xlsx
@@ -11090,13 +11090,13 @@
         <v>Redes TCP/IP Intermediário</v>
       </c>
       <c r="H334">
-        <v>78.95</v>
+        <v>100</v>
       </c>
       <c r="I334">
-        <v>28</v>
-      </c>
-      <c r="J334" t="str">
-        <v>Pendente</v>
+        <v>61</v>
+      </c>
+      <c r="J334">
+        <v>70</v>
       </c>
     </row>
     <row r="335">
@@ -11122,13 +11122,13 @@
         <v>Redes TCP/IP Intermediário</v>
       </c>
       <c r="H335">
-        <v>78.95</v>
+        <v>100</v>
       </c>
       <c r="I335">
-        <v>28</v>
-      </c>
-      <c r="J335" t="str">
-        <v>Pendente</v>
+        <v>61</v>
+      </c>
+      <c r="J335">
+        <v>70</v>
       </c>
     </row>
     <row r="336">
@@ -11154,13 +11154,13 @@
         <v>Redes TCP/IP Intermediário</v>
       </c>
       <c r="H336">
-        <v>78.95</v>
+        <v>100</v>
       </c>
       <c r="I336">
-        <v>28</v>
-      </c>
-      <c r="J336" t="str">
-        <v>Pendente</v>
+        <v>61</v>
+      </c>
+      <c r="J336">
+        <v>70</v>
       </c>
     </row>
     <row r="337">
@@ -11186,10 +11186,10 @@
         <v>Redes TCP/IP Avançado</v>
       </c>
       <c r="H337">
-        <v>0</v>
+        <v>26.32</v>
       </c>
       <c r="I337">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="J337" t="str">
         <v>Pendente</v>
@@ -11218,10 +11218,10 @@
         <v>Redes TCP/IP Avançado</v>
       </c>
       <c r="H338">
-        <v>0</v>
+        <v>26.32</v>
       </c>
       <c r="I338">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="J338" t="str">
         <v>Pendente</v>

</xml_diff>